<commit_message>
IMPLEMENTACION DE METODOS Y SERVICIOS PARA RECUPERAR PROVEEDOR CON IDENTIFICADOR || RETO 16 SERVICIOS VARIOS ||funciona ok
</commit_message>
<xml_diff>
--- a/Base de Datos/01DiseñoBDD.xlsx
+++ b/Base de Datos/01DiseñoBDD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ESCUELAPROGRAMACIONKD\03MODULO\inventarios\Base de Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82CD2806-7FD2-49F4-AEB6-43A16E1F6204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABEF119-62E1-44CC-BF90-98B8269B0AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E9E292EC-47DE-4FD1-BDC6-A5B6D9350F58}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9E292EC-47DE-4FD1-BDC6-A5B6D9350F58}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLAS BDD" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="137">
   <si>
     <t>CATEGORIAS</t>
   </si>
@@ -442,6 +442,15 @@
   </si>
   <si>
     <t>Recupera los pedidos con sus respectivos detalles de un proveedor determinado. Recibe el identificador del proveedor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET </t>
+  </si>
+  <si>
+    <t>/provedores/buscar/{identificador]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">recupera el rpoveedor, recibe el indenficador del proveedor como parametro </t>
   </si>
 </sst>
 </file>
@@ -789,28 +798,28 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1171,11 +1180,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="8" t="s">
@@ -1266,15 +1275,15 @@
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="43"/>
+      <c r="D12" s="41"/>
       <c r="E12" s="42"/>
-      <c r="G12" s="44" t="s">
+      <c r="G12" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="44"/>
+      <c r="H12" s="39"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C13" s="8" t="s">
@@ -1395,16 +1404,16 @@
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
@@ -1537,10 +1546,10 @@
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C31" s="44" t="s">
+      <c r="C31" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="D31" s="44"/>
+      <c r="D31" s="39"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C32" s="8" t="s">
@@ -1567,14 +1576,14 @@
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="44" t="s">
+      <c r="B36" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="44"/>
-      <c r="D36" s="44"/>
-      <c r="E36" s="44"/>
-      <c r="F36" s="44"/>
-      <c r="G36" s="44"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="8" t="s">
@@ -1637,13 +1646,13 @@
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="45" t="s">
+      <c r="B42" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="I42" s="41" t="s">
+      <c r="C42" s="44"/>
+      <c r="D42" s="44"/>
+      <c r="E42" s="44"/>
+      <c r="I42" s="40" t="s">
         <v>80</v>
       </c>
       <c r="J42" s="42"/>
@@ -1709,14 +1718,14 @@
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="44" t="s">
+      <c r="B47" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="44"/>
-      <c r="D47" s="44"/>
-      <c r="E47" s="44"/>
-      <c r="F47" s="44"/>
-      <c r="G47" s="44"/>
+      <c r="C47" s="39"/>
+      <c r="D47" s="39"/>
+      <c r="E47" s="39"/>
+      <c r="F47" s="39"/>
+      <c r="G47" s="39"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
@@ -1807,12 +1816,12 @@
       <c r="G52" s="2"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B54" s="41" t="s">
+      <c r="B54" s="40" t="s">
         <v>85</v>
       </c>
-      <c r="C54" s="43"/>
-      <c r="D54" s="43"/>
-      <c r="E54" s="43"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="41"/>
       <c r="F54" s="42"/>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.25">
@@ -1927,12 +1936,12 @@
       </c>
     </row>
     <row r="64" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B64" s="41" t="s">
+      <c r="B64" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="C64" s="43"/>
-      <c r="D64" s="43"/>
-      <c r="E64" s="43"/>
+      <c r="C64" s="41"/>
+      <c r="D64" s="41"/>
+      <c r="E64" s="41"/>
       <c r="F64" s="42"/>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
@@ -1970,15 +1979,15 @@
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B69" s="39" t="s">
+      <c r="B69" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="C69" s="40"/>
-      <c r="D69" s="40"/>
-      <c r="E69" s="40"/>
-      <c r="F69" s="40"/>
-      <c r="G69" s="40"/>
-      <c r="H69" s="40"/>
+      <c r="C69" s="46"/>
+      <c r="D69" s="46"/>
+      <c r="E69" s="46"/>
+      <c r="F69" s="46"/>
+      <c r="G69" s="46"/>
+      <c r="H69" s="46"/>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="8" t="s">
@@ -2072,11 +2081,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="B47:G47"/>
-    <mergeCell ref="B42:E42"/>
     <mergeCell ref="B69:H69"/>
     <mergeCell ref="I42:J42"/>
     <mergeCell ref="B23:I23"/>
@@ -2084,6 +2088,11 @@
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="B47:G47"/>
+    <mergeCell ref="B42:E42"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
@@ -2269,9 +2278,15 @@
       <c r="E16" s="37"/>
     </row>
     <row r="17" spans="2:4" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
+      <c r="B17" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="D17" s="36" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="18" spans="2:4" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B18" s="36"/>

</xml_diff>

<commit_message>
IMPLEMENTACION DE METODOS Y SERVICIOS PARA RECUPERAR PRODUCTO CON IDENTIFICADOR || RETO 16 SERVICIOS VARIOS ||funciona ok
</commit_message>
<xml_diff>
--- a/Base de Datos/01DiseñoBDD.xlsx
+++ b/Base de Datos/01DiseñoBDD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ESCUELAPROGRAMACIONKD\03MODULO\inventarios\Base de Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABEF119-62E1-44CC-BF90-98B8269B0AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102629CE-0F9F-4A55-A3E5-AE9882FCCFFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9E292EC-47DE-4FD1-BDC6-A5B6D9350F58}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E9E292EC-47DE-4FD1-BDC6-A5B6D9350F58}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLAS BDD" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="141">
   <si>
     <t>CATEGORIAS</t>
   </si>
@@ -447,10 +447,22 @@
     <t xml:space="preserve">GET </t>
   </si>
   <si>
-    <t>/provedores/buscar/{identificador]</t>
-  </si>
-  <si>
     <t xml:space="preserve">recupera el rpoveedor, recibe el indenficador del proveedor como parametro </t>
+  </si>
+  <si>
+    <t>/provedores/recuperar/{identificador}</t>
+  </si>
+  <si>
+    <t>/productos/recuperar/{identificador}</t>
+  </si>
+  <si>
+    <t>recupera el producto recibe el didentificador del producto.</t>
+  </si>
+  <si>
+    <t>NOMBRE PK</t>
+  </si>
+  <si>
+    <t>reto 16</t>
   </si>
 </sst>
 </file>
@@ -526,7 +538,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -602,6 +614,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -700,7 +718,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -794,10 +812,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -824,6 +838,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1180,11 +1203,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="8" t="s">
@@ -1275,19 +1298,19 @@
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C12" s="40" t="s">
+      <c r="C12" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="41"/>
-      <c r="E12" s="42"/>
-      <c r="G12" s="39" t="s">
+      <c r="D12" s="39"/>
+      <c r="E12" s="40"/>
+      <c r="G12" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="39"/>
+      <c r="H12" s="37"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C13" s="8" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>23</v>
@@ -1404,16 +1427,16 @@
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
@@ -1546,10 +1569,10 @@
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C31" s="39" t="s">
+      <c r="C31" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="D31" s="39"/>
+      <c r="D31" s="37"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C32" s="8" t="s">
@@ -1576,14 +1599,14 @@
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="39" t="s">
+      <c r="B36" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="8" t="s">
@@ -1646,16 +1669,16 @@
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="43" t="s">
+      <c r="B42" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="44"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="44"/>
-      <c r="I42" s="40" t="s">
+      <c r="C42" s="42"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="42"/>
+      <c r="I42" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="J42" s="42"/>
+      <c r="J42" s="40"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
@@ -1718,14 +1741,14 @@
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="39" t="s">
+      <c r="B47" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="39"/>
-      <c r="D47" s="39"/>
-      <c r="E47" s="39"/>
-      <c r="F47" s="39"/>
-      <c r="G47" s="39"/>
+      <c r="C47" s="37"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
@@ -1816,13 +1839,13 @@
       <c r="G52" s="2"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B54" s="40" t="s">
+      <c r="B54" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="C54" s="41"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="41"/>
-      <c r="F54" s="42"/>
+      <c r="C54" s="39"/>
+      <c r="D54" s="39"/>
+      <c r="E54" s="39"/>
+      <c r="F54" s="40"/>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="8" t="s">
@@ -1936,13 +1959,13 @@
       </c>
     </row>
     <row r="64" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B64" s="40" t="s">
+      <c r="B64" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="C64" s="41"/>
-      <c r="D64" s="41"/>
-      <c r="E64" s="41"/>
-      <c r="F64" s="42"/>
+      <c r="C64" s="39"/>
+      <c r="D64" s="39"/>
+      <c r="E64" s="39"/>
+      <c r="F64" s="40"/>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="8" t="s">
@@ -1979,15 +2002,15 @@
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B69" s="45" t="s">
+      <c r="B69" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="C69" s="46"/>
-      <c r="D69" s="46"/>
-      <c r="E69" s="46"/>
-      <c r="F69" s="46"/>
-      <c r="G69" s="46"/>
-      <c r="H69" s="46"/>
+      <c r="C69" s="44"/>
+      <c r="D69" s="44"/>
+      <c r="E69" s="44"/>
+      <c r="F69" s="44"/>
+      <c r="G69" s="44"/>
+      <c r="H69" s="44"/>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="8" t="s">
@@ -2113,14 +2136,15 @@
     <col min="2" max="2" width="16.140625" style="33" customWidth="1"/>
     <col min="3" max="3" width="52.140625" style="33" customWidth="1"/>
     <col min="4" max="4" width="138.85546875" style="33" customWidth="1"/>
+    <col min="5" max="5" width="31.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
     </row>
     <row r="3" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
@@ -2222,80 +2246,95 @@
       </c>
     </row>
     <row r="12" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="46" t="s">
         <v>124</v>
       </c>
-      <c r="D12" s="36" t="s">
+      <c r="D12" s="46" t="s">
         <v>125</v>
       </c>
+      <c r="E12" s="48" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="13" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="46" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="36" t="s">
+      <c r="C13" s="46" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="47" t="s">
         <v>127</v>
       </c>
+      <c r="E13" s="48"/>
     </row>
     <row r="14" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C14" s="36" t="s">
+      <c r="C14" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="D14" s="36" t="s">
+      <c r="D14" s="46" t="s">
         <v>129</v>
       </c>
+      <c r="E14" s="48"/>
     </row>
     <row r="15" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="36" t="s">
+      <c r="C15" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="D15" s="36" t="s">
+      <c r="D15" s="46" t="s">
         <v>131</v>
       </c>
+      <c r="E15" s="48"/>
     </row>
     <row r="16" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="C16" s="36" t="s">
+      <c r="C16" s="46" t="s">
         <v>132</v>
       </c>
-      <c r="D16" s="36" t="s">
+      <c r="D16" s="46" t="s">
         <v>133</v>
       </c>
-      <c r="E16" s="37"/>
-    </row>
-    <row r="17" spans="2:4" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B17" s="36" t="s">
+      <c r="E16" s="48"/>
+    </row>
+    <row r="17" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B17" s="46" t="s">
         <v>134</v>
       </c>
-      <c r="C17" s="36" t="s">
+      <c r="C17" s="46" t="s">
+        <v>136</v>
+      </c>
+      <c r="D17" s="46" t="s">
         <v>135</v>
       </c>
-      <c r="D17" s="36" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
+      <c r="E17" s="48"/>
+    </row>
+    <row r="18" spans="2:5" s="35" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B18" s="46" t="s">
+        <v>134</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>137</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>138</v>
+      </c>
+      <c r="E18" s="48"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E12:E18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="0" r:id="rId1"/>

</xml_diff>